<commit_message>
Latest data: Mon Sep 14 17:29:00 UTC 2026
</commit_message>
<xml_diff>
--- a/docs/particelle_non_trovate.xlsx
+++ b/docs/particelle_non_trovate.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -693,11 +693,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>3597/16</t>
+          <t>878</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>9</v>
+        <v>134</v>
       </c>
     </row>
     <row r="22">
@@ -706,11 +706,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>3597/18</t>
+          <t>879</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>9</v>
+        <v>134</v>
       </c>
     </row>
     <row r="23">
@@ -719,11 +719,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>3597/22</t>
+          <t>880</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>9</v>
+        <v>134</v>
       </c>
     </row>
     <row r="24">
@@ -732,11 +732,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>3697</t>
+          <t>881</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>9</v>
+        <v>134</v>
       </c>
     </row>
     <row r="25">
@@ -745,11 +745,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2331/38</t>
+          <t>885/2</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>258</v>
+        <v>134</v>
       </c>
     </row>
     <row r="26">
@@ -758,11 +758,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2068/43</t>
+          <t>.71</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>310</v>
+        <v>134</v>
       </c>
     </row>
     <row r="27">
@@ -771,11 +771,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2822/12</t>
+          <t>.72</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>310</v>
+        <v>134</v>
       </c>
     </row>
     <row r="28">
@@ -784,11 +784,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2822/16</t>
+          <t>.73</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>310</v>
+        <v>134</v>
       </c>
     </row>
     <row r="29">
@@ -797,11 +797,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2020/14</t>
+          <t>.74</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>310</v>
+        <v>134</v>
       </c>
     </row>
     <row r="30">
@@ -810,11 +810,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>.384</t>
+          <t>3597/16</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>139</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31">
@@ -823,11 +823,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>766</t>
+          <t>3597/18</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>140</v>
+        <v>9</v>
       </c>
     </row>
     <row r="32">
@@ -836,11 +836,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>.1512</t>
+          <t>3597/22</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>140</v>
+        <v>9</v>
       </c>
     </row>
     <row r="33">
@@ -849,11 +849,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>.7.</t>
+          <t>3697</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>187</v>
+        <v>9</v>
       </c>
     </row>
     <row r="34">
@@ -862,11 +862,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2727/1</t>
+          <t>2331/38</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>189</v>
+        <v>258</v>
       </c>
     </row>
     <row r="35">
@@ -875,11 +875,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>47/3</t>
+          <t>2068/43</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>277</v>
+        <v>310</v>
       </c>
     </row>
     <row r="36">
@@ -888,11 +888,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>302/1</t>
+          <t>2822/12</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>277</v>
+        <v>310</v>
       </c>
     </row>
     <row r="37">
@@ -901,11 +901,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2103/7</t>
+          <t>2822/16</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>394</v>
+        <v>310</v>
       </c>
     </row>
     <row r="38">
@@ -914,11 +914,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>.4047</t>
+          <t>2020/14</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="39">
@@ -927,11 +927,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>.4046</t>
+          <t>.384</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>307</v>
+        <v>139</v>
       </c>
     </row>
     <row r="40">
@@ -940,10 +940,127 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
+          <t>766</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>.1512</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>.7.</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2727/1</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>47/3</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>302/1</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2103/7</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>.4047</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>.4046</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
           <t>1064/3</t>
         </is>
       </c>
-      <c r="C40" t="n">
+      <c r="C49" t="n">
         <v>248</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Latest data: Mon Sep 14 22:59:51 UTC 2026
</commit_message>
<xml_diff>
--- a/docs/particelle_non_trovate.xlsx
+++ b/docs/particelle_non_trovate.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -693,11 +693,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>878</t>
+          <t>3597/16</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>134</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22">
@@ -706,11 +706,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>879</t>
+          <t>3597/18</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>134</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23">
@@ -719,11 +719,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>880</t>
+          <t>3597/22</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>134</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24">
@@ -732,11 +732,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>881</t>
+          <t>3697</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>134</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25">
@@ -745,11 +745,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>885/2</t>
+          <t>2331/38</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>134</v>
+        <v>258</v>
       </c>
     </row>
     <row r="26">
@@ -758,11 +758,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>.71</t>
+          <t>2068/43</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>134</v>
+        <v>310</v>
       </c>
     </row>
     <row r="27">
@@ -771,11 +771,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>.72</t>
+          <t>2822/12</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>134</v>
+        <v>310</v>
       </c>
     </row>
     <row r="28">
@@ -784,11 +784,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>.73</t>
+          <t>2822/16</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>134</v>
+        <v>310</v>
       </c>
     </row>
     <row r="29">
@@ -797,11 +797,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>.74</t>
+          <t>2020/14</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>134</v>
+        <v>310</v>
       </c>
     </row>
     <row r="30">
@@ -810,11 +810,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>3597/16</t>
+          <t>.384</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>9</v>
+        <v>139</v>
       </c>
     </row>
     <row r="31">
@@ -823,11 +823,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>3597/18</t>
+          <t>766</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>9</v>
+        <v>140</v>
       </c>
     </row>
     <row r="32">
@@ -836,11 +836,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>3597/22</t>
+          <t>.1512</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>9</v>
+        <v>140</v>
       </c>
     </row>
     <row r="33">
@@ -849,11 +849,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>3697</t>
+          <t>.7.</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>9</v>
+        <v>187</v>
       </c>
     </row>
     <row r="34">
@@ -862,11 +862,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2331/38</t>
+          <t>2727/1</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>258</v>
+        <v>189</v>
       </c>
     </row>
     <row r="35">
@@ -875,11 +875,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2068/43</t>
+          <t>47/3</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>310</v>
+        <v>277</v>
       </c>
     </row>
     <row r="36">
@@ -888,11 +888,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2822/12</t>
+          <t>302/1</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>310</v>
+        <v>277</v>
       </c>
     </row>
     <row r="37">
@@ -901,11 +901,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2822/16</t>
+          <t>2103/7</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>310</v>
+        <v>394</v>
       </c>
     </row>
     <row r="38">
@@ -914,11 +914,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2020/14</t>
+          <t>.4047</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="39">
@@ -927,11 +927,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>.384</t>
+          <t>.4046</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>139</v>
+        <v>307</v>
       </c>
     </row>
     <row r="40">
@@ -940,127 +940,10 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>766</t>
+          <t>1064/3</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="1" t="n">
-        <v>39</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>.1512</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="1" t="n">
-        <v>40</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>.7.</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="1" t="n">
-        <v>41</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>2727/1</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="1" t="n">
-        <v>42</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>47/3</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="1" t="n">
-        <v>43</v>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>302/1</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="1" t="n">
-        <v>44</v>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>2103/7</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="1" t="n">
-        <v>45</v>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>.4047</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="1" t="n">
-        <v>46</v>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>.4046</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="1" t="n">
-        <v>47</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>1064/3</t>
-        </is>
-      </c>
-      <c r="C49" t="n">
         <v>248</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Latest data: Wed Oct 21 23:01:25 UTC 2026
</commit_message>
<xml_diff>
--- a/docs/particelle_non_trovate.xlsx
+++ b/docs/particelle_non_trovate.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -628,11 +628,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1115</t>
+          <t>759</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>7</v>
+        <v>230</v>
       </c>
     </row>
     <row r="17">
@@ -641,11 +641,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>.451</t>
+          <t>864/6</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>88</v>
+        <v>230</v>
       </c>
     </row>
     <row r="18">
@@ -654,11 +654,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>274</t>
+          <t>864/10</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>202</v>
+        <v>230</v>
       </c>
     </row>
     <row r="19">
@@ -667,11 +667,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1341</t>
+          <t>867/2</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>132</v>
+        <v>230</v>
       </c>
     </row>
     <row r="20">
@@ -680,11 +680,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>703</t>
+          <t>867/3</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>61</v>
+        <v>230</v>
       </c>
     </row>
     <row r="21">
@@ -693,11 +693,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>3597/16</t>
+          <t>929/3</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>9</v>
+        <v>230</v>
       </c>
     </row>
     <row r="22">
@@ -706,11 +706,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>3597/18</t>
+          <t>929/73</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>9</v>
+        <v>230</v>
       </c>
     </row>
     <row r="23">
@@ -719,11 +719,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>3597/22</t>
+          <t>929/88</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>9</v>
+        <v>230</v>
       </c>
     </row>
     <row r="24">
@@ -732,11 +732,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>3697</t>
+          <t>938/1</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>9</v>
+        <v>230</v>
       </c>
     </row>
     <row r="25">
@@ -745,11 +745,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2331/38</t>
+          <t>938/3</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>258</v>
+        <v>230</v>
       </c>
     </row>
     <row r="26">
@@ -758,11 +758,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2068/43</t>
+          <t>938/13</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>310</v>
+        <v>230</v>
       </c>
     </row>
     <row r="27">
@@ -771,11 +771,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2822/12</t>
+          <t>938/21</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>310</v>
+        <v>230</v>
       </c>
     </row>
     <row r="28">
@@ -784,11 +784,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2822/16</t>
+          <t>938/42</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>310</v>
+        <v>230</v>
       </c>
     </row>
     <row r="29">
@@ -797,11 +797,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2020/14</t>
+          <t>938/66</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>310</v>
+        <v>230</v>
       </c>
     </row>
     <row r="30">
@@ -810,11 +810,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>.384</t>
+          <t>938/67</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>139</v>
+        <v>230</v>
       </c>
     </row>
     <row r="31">
@@ -823,11 +823,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>766</t>
+          <t>940/2</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>140</v>
+        <v>230</v>
       </c>
     </row>
     <row r="32">
@@ -836,11 +836,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>.1512</t>
+          <t>941</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>140</v>
+        <v>230</v>
       </c>
     </row>
     <row r="33">
@@ -849,11 +849,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>.7.</t>
+          <t>942/1</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>187</v>
+        <v>230</v>
       </c>
     </row>
     <row r="34">
@@ -862,11 +862,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2727/1</t>
+          <t>942/2</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>189</v>
+        <v>230</v>
       </c>
     </row>
     <row r="35">
@@ -875,11 +875,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>47/3</t>
+          <t>943</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>277</v>
+        <v>230</v>
       </c>
     </row>
     <row r="36">
@@ -888,11 +888,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>302/1</t>
+          <t>944</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>277</v>
+        <v>230</v>
       </c>
     </row>
     <row r="37">
@@ -901,11 +901,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2103/7</t>
+          <t>945/6</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>394</v>
+        <v>230</v>
       </c>
     </row>
     <row r="38">
@@ -914,11 +914,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>.4047</t>
+          <t>945/7</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>307</v>
+        <v>230</v>
       </c>
     </row>
     <row r="39">
@@ -927,11 +927,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>.4046</t>
+          <t>947/15</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>307</v>
+        <v>230</v>
       </c>
     </row>
     <row r="40">
@@ -940,10 +940,1804 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
+          <t>947/43</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>947/67</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>947/100</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>947/104</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>947/125</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>948/1</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>948/68</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1353/1</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1353/32</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1373</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1374</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1378/2</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1378/3</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>1382</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1383</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1384</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>1385</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="n">
+        <v>55</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>1386</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1387/3</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="n">
+        <v>57</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>1402/2</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="n">
+        <v>58</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1403/2</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="n">
+        <v>59</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>1404/2</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>1405/2</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1406/2</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="n">
+        <v>62</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1408/2</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="n">
+        <v>63</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>1409/1</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="n">
+        <v>64</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>1410</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>1411/1</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="n">
+        <v>66</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>1411/2</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
+        <v>67</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>1411/3</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="n">
+        <v>68</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>1411/4</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="n">
+        <v>69</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>1412</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="n">
+        <v>70</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>1414</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="n">
+        <v>71</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>1419</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="n">
+        <v>72</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>1420</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="n">
+        <v>73</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>1421/3</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="n">
+        <v>74</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>1423</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="n">
+        <v>75</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>1424/2</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="n">
+        <v>76</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>1424/3</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="n">
+        <v>77</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>1424/13</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="n">
+        <v>78</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>1424/14</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="n">
+        <v>79</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>1425</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>1427</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="n">
+        <v>81</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>1428</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="n">
+        <v>82</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>1429</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="1" t="n">
+        <v>83</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>1430</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="1" t="n">
+        <v>84</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>1446/2</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="1" t="n">
+        <v>85</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>1448/2</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="1" t="n">
+        <v>86</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>1471/12</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="1" t="n">
+        <v>87</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>1471/4</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>1474</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="1" t="n">
+        <v>89</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>1475</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1478/1</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="1" t="n">
+        <v>91</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1478/2</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1479/1</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="1" t="n">
+        <v>93</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>1479/2</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="1" t="n">
+        <v>94</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>1487/1</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="1" t="n">
+        <v>95</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>1487/8</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="1" t="n">
+        <v>96</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>1487/9</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="1" t="n">
+        <v>97</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>1487/10</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="1" t="n">
+        <v>98</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>1487/11</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="1" t="n">
+        <v>99</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1487/12</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>1488/1</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="1" t="n">
+        <v>101</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1488/2</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="1" t="n">
+        <v>102</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1488/3</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="1" t="n">
+        <v>103</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>1488/6</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="1" t="n">
+        <v>104</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1488/7</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="1" t="n">
+        <v>105</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>1502/3</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="1" t="n">
+        <v>106</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>1509/2</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="1" t="n">
+        <v>107</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>1510/2</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="1" t="n">
+        <v>108</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>1527</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="1" t="n">
+        <v>109</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>1530/1</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="1" t="n">
+        <v>110</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>1578/1</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="1" t="n">
+        <v>111</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>1578/11</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="1" t="n">
+        <v>112</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>1578/12</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="1" t="n">
+        <v>113</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>1578/14</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="1" t="n">
+        <v>114</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>1578/19</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="1" t="n">
+        <v>115</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>1578/20</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="1" t="n">
+        <v>116</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1592/1</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="1" t="n">
+        <v>117</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>1593/1</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="1" t="n">
+        <v>118</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>1594/1</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="1" t="n">
+        <v>119</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1594/15</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="1" t="n">
+        <v>120</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>1595/1</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="1" t="n">
+        <v>121</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>1596/1</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="1" t="n">
+        <v>122</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1596/20</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="1" t="n">
+        <v>123</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1597/1</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="1" t="n">
+        <v>124</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1597/1</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="1" t="n">
+        <v>125</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>1597/5</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="1" t="n">
+        <v>126</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>1598/1</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="1" t="n">
+        <v>127</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>1599/1</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="1" t="n">
+        <v>128</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>1602/4</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="1" t="n">
+        <v>129</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>1603/4</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="1" t="n">
+        <v>130</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>1604/3</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="1" t="n">
+        <v>131</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>1609</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="1" t="n">
+        <v>132</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>1705/1</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="1" t="n">
+        <v>133</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>1705/2</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="1" t="n">
+        <v>134</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>1705/5</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="1" t="n">
+        <v>135</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>1706/1</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="1" t="n">
+        <v>136</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>1708/3</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="1" t="n">
+        <v>137</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>1709/2</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="1" t="n">
+        <v>138</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>1726/1</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="1" t="n">
+        <v>139</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>1727</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="1" t="n">
+        <v>140</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>1735</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="1" t="n">
+        <v>141</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>1738</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="1" t="n">
+        <v>142</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>1840</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="1" t="n">
+        <v>143</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>2027/1</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="1" t="n">
+        <v>144</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>2027/2</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="1" t="n">
+        <v>145</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>.176/3</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="1" t="n">
+        <v>146</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>.176/4</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="1" t="n">
+        <v>147</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>.176/5</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="1" t="n">
+        <v>148</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>.307</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="1" t="n">
+        <v>149</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>.361</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="1" t="n">
+        <v>150</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>.988</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="1" t="n">
+        <v>151</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>.1053</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="1" t="n">
+        <v>152</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>1115</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="1" t="n">
+        <v>153</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>.451</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="1" t="n">
+        <v>154</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>274</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="1" t="n">
+        <v>155</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>1341</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="1" t="n">
+        <v>156</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>703</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="1" t="n">
+        <v>157</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>3597/16</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="1" t="n">
+        <v>158</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>3597/18</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="1" t="n">
+        <v>159</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>3597/22</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="1" t="n">
+        <v>160</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>3697</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="1" t="n">
+        <v>161</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>2331/38</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="1" t="n">
+        <v>162</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>2068/43</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="1" t="n">
+        <v>163</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>2822/12</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="1" t="n">
+        <v>164</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>2822/16</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="1" t="n">
+        <v>165</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>2020/14</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="1" t="n">
+        <v>166</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>.384</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="1" t="n">
+        <v>167</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>766</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="1" t="n">
+        <v>168</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>.1512</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="1" t="n">
+        <v>169</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>.7.</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="1" t="n">
+        <v>170</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>2727/1</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="1" t="n">
+        <v>171</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>47/3</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="1" t="n">
+        <v>172</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>302/1</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="1" t="n">
+        <v>173</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>2103/7</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="1" t="n">
+        <v>174</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>.4047</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="1" t="n">
+        <v>175</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>.4046</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="1" t="n">
+        <v>176</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
           <t>1064/3</t>
         </is>
       </c>
-      <c r="C40" t="n">
+      <c r="C178" t="n">
         <v>248</v>
       </c>
     </row>

</xml_diff>